<commit_message>
petit changement projet navajo
</commit_message>
<xml_diff>
--- a/public/2026 E5 - TS SISR.xlsx
+++ b/public/2026 E5 - TS SISR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roblo\Desktop\portfolio\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8713C0-59F7-452F-97B8-957C4BB7DF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960EFA31-DFAE-455E-8776-A85D315B631A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -170,9 +170,6 @@
     <t>Présence en ligne du SDIS 33</t>
   </si>
   <si>
-    <t>Gestion de l'identité professionnel</t>
-  </si>
-  <si>
     <t>9/2/2026
 20/02/2026</t>
   </si>
@@ -183,6 +180,9 @@
   <si>
     <t>10/12/2025
 28/01/2026</t>
+  </si>
+  <si>
+    <t>Gestion de l'identité professionnelle</t>
   </si>
 </sst>
 </file>
@@ -711,16 +711,20 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -742,15 +746,11 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1082,40 +1082,40 @@
       <c r="B5" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="41" t="s">
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="42"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="41" t="s">
+      <c r="J5" s="45"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="42"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="41" t="s">
+      <c r="M5" s="45"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="P5" s="42"/>
-      <c r="Q5" s="43"/>
-      <c r="R5" s="41" t="s">
+      <c r="P5" s="45"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="S5" s="42"/>
-      <c r="T5" s="43"/>
-      <c r="U5" s="41" t="s">
+      <c r="S5" s="45"/>
+      <c r="T5" s="46"/>
+      <c r="U5" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="V5" s="42"/>
-      <c r="W5" s="42"/>
-      <c r="X5" s="43"/>
+      <c r="V5" s="45"/>
+      <c r="W5" s="45"/>
+      <c r="X5" s="46"/>
     </row>
     <row r="6" spans="1:26" ht="324.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="54"/>
@@ -1190,32 +1190,32 @@
       <c r="Z6" s="8"/>
     </row>
     <row r="7" spans="1:26" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="57" t="s">
+      <c r="A7" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
-      <c r="U7" s="45"/>
-      <c r="V7" s="45"/>
-      <c r="W7" s="45"/>
-      <c r="X7" s="46"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="58"/>
+      <c r="K7" s="58"/>
+      <c r="L7" s="58"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="58"/>
+      <c r="R7" s="58"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="58"/>
+      <c r="X7" s="59"/>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
     </row>
@@ -1224,7 +1224,7 @@
         <v>38</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
@@ -1256,7 +1256,7 @@
         <v>39</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="21"/>
@@ -1287,7 +1287,7 @@
       <c r="A10" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="59">
+      <c r="B10" s="42">
         <v>2025</v>
       </c>
       <c r="C10" s="32"/>
@@ -1316,16 +1316,16 @@
       <c r="Z10" s="8"/>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="46"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58"/>
+      <c r="H11" s="59"/>
       <c r="I11" s="23"/>
       <c r="J11" s="24"/>
       <c r="K11" s="25"/>
@@ -1402,16 +1402,16 @@
       <c r="Z13" s="8"/>
     </row>
     <row r="14" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
+      <c r="B14" s="58"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="59"/>
       <c r="I14" s="23"/>
       <c r="J14" s="24"/>
       <c r="K14" s="25"/>
@@ -1435,7 +1435,7 @@
       <c r="A15" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="58">
+      <c r="B15" s="41">
         <v>45818</v>
       </c>
       <c r="C15" s="20"/>
@@ -1467,8 +1467,8 @@
       <c r="A16" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="60" t="s">
-        <v>47</v>
+      <c r="B16" s="43" t="s">
+        <v>46</v>
       </c>
       <c r="C16" s="36"/>
       <c r="D16" s="21"/>
@@ -1499,7 +1499,7 @@
       <c r="A17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="58">
+      <c r="B17" s="41">
         <v>46115</v>
       </c>
       <c r="C17" s="20"/>
@@ -1529,9 +1529,9 @@
     </row>
     <row r="18" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
-      <c r="B18" s="58">
+      <c r="B18" s="41">
         <v>46084</v>
       </c>
       <c r="C18" s="20"/>
@@ -11229,6 +11229,10 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="A7:X7"/>
     <mergeCell ref="O5:Q5"/>
     <mergeCell ref="R5:T5"/>
     <mergeCell ref="U5:X5"/>
@@ -11241,10 +11245,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="A7:X7"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.1" bottom="0.1" header="0.3" footer="0.3"/>

</xml_diff>